<commit_message>
Actualizacion BD pesos frescos y agregacion
</commit_message>
<xml_diff>
--- a/BD Cobre.xlsx
+++ b/BD Cobre.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julip\GitHub\Cobre\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534E204F-2FE7-4665-93E8-8CE91BE81CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11040"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="58">
   <si>
     <t>id</t>
   </si>
@@ -106,12 +100,105 @@
   </si>
   <si>
     <t>CuVastago</t>
+  </si>
+  <si>
+    <t>pf raiz</t>
+  </si>
+  <si>
+    <t>p seco raiz</t>
+  </si>
+  <si>
+    <t>largo vasta</t>
+  </si>
+  <si>
+    <t>pf aer</t>
+  </si>
+  <si>
+    <t>p s aereo</t>
+  </si>
+  <si>
+    <t>RAIZ+TIERRA</t>
+  </si>
+  <si>
+    <t>adherido</t>
+  </si>
+  <si>
+    <t>506,21</t>
+  </si>
+  <si>
+    <t>166,65</t>
+  </si>
+  <si>
+    <t>330,50</t>
+  </si>
+  <si>
+    <t>317,26</t>
+  </si>
+  <si>
+    <t>151,55</t>
+  </si>
+  <si>
+    <t>202,84</t>
+  </si>
+  <si>
+    <t>553,50</t>
+  </si>
+  <si>
+    <t>510,23</t>
+  </si>
+  <si>
+    <t>499,54</t>
+  </si>
+  <si>
+    <t>602,80</t>
+  </si>
+  <si>
+    <t>451,20</t>
+  </si>
+  <si>
+    <t>646,10</t>
+  </si>
+  <si>
+    <t>283,64</t>
+  </si>
+  <si>
+    <t>512,02</t>
+  </si>
+  <si>
+    <t>232,64</t>
+  </si>
+  <si>
+    <t>298,00</t>
+  </si>
+  <si>
+    <t>219,90</t>
+  </si>
+  <si>
+    <t>495,33</t>
+  </si>
+  <si>
+    <t>748,86</t>
+  </si>
+  <si>
+    <t>426,74</t>
+  </si>
+  <si>
+    <t>569,88</t>
+  </si>
+  <si>
+    <t>342,04</t>
+  </si>
+  <si>
+    <t>198,64</t>
+  </si>
+  <si>
+    <t>366,62</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -239,7 +326,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -574,12 +661,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="169">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1074,10 +1185,13 @@
     <xf numFmtId="2" fontId="4" fillId="14" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{D6A77139-65C8-49F1-9AB5-DA957D2A9824}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1135,7 +1249,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1170,7 +1284,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1347,21 +1461,21 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X43"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AE43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1434,8 +1548,29 @@
       <c r="X1" s="6" t="s">
         <v>23</v>
       </c>
+      <c r="Y1" s="166" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="166" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA1" s="166" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB1" s="166" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC1" s="166" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD1" s="167" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE1" s="168" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1491,7 +1626,7 @@
       <c r="W2" s="9"/>
       <c r="X2" s="11"/>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1533,7 +1668,7 @@
       <c r="W3" s="14"/>
       <c r="X3" s="15"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1575,7 +1710,7 @@
       <c r="W4" s="14"/>
       <c r="X4" s="15"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1631,7 +1766,7 @@
       <c r="W5" s="18"/>
       <c r="X5" s="20"/>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1687,7 +1822,7 @@
       <c r="W6" s="18"/>
       <c r="X6" s="20"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1743,7 +1878,7 @@
       <c r="W7" s="18"/>
       <c r="X7" s="20"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1799,7 +1934,7 @@
       <c r="W8" s="25"/>
       <c r="X8" s="26"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1855,7 +1990,7 @@
       <c r="W9" s="25"/>
       <c r="X9" s="26"/>
     </row>
-    <row r="10" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1911,7 +2046,7 @@
       <c r="W10" s="29"/>
       <c r="X10" s="30"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1971,7 +2106,7 @@
       <c r="W11" s="34"/>
       <c r="X11" s="36"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2031,7 +2166,7 @@
       <c r="W12" s="40"/>
       <c r="X12" s="42"/>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2073,7 +2208,7 @@
       <c r="W13" s="40"/>
       <c r="X13" s="42"/>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -2133,7 +2268,7 @@
       <c r="W14" s="46"/>
       <c r="X14" s="48"/>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -2193,7 +2328,7 @@
       <c r="W15" s="46"/>
       <c r="X15" s="48"/>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -2251,7 +2386,7 @@
       <c r="W16" s="46"/>
       <c r="X16" s="48"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -2311,7 +2446,7 @@
       <c r="W17" s="53"/>
       <c r="X17" s="55"/>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -2371,7 +2506,7 @@
       <c r="W18" s="53"/>
       <c r="X18" s="55"/>
     </row>
-    <row r="19" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -2431,7 +2566,7 @@
       <c r="W19" s="60"/>
       <c r="X19" s="62"/>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -2490,8 +2625,30 @@
       <c r="X20" s="69">
         <v>100</v>
       </c>
+      <c r="Y20" s="69">
+        <v>5.5</v>
+      </c>
+      <c r="Z20" s="69">
+        <v>1.1176999999999999</v>
+      </c>
+      <c r="AA20" s="69">
+        <v>134</v>
+      </c>
+      <c r="AB20" s="69">
+        <f>66.01+0.26</f>
+        <v>66.27000000000001</v>
+      </c>
+      <c r="AC20" s="69">
+        <v>12.5967</v>
+      </c>
+      <c r="AD20" s="69">
+        <v>1565.5</v>
+      </c>
+      <c r="AE20" s="69" t="s">
+        <v>46</v>
+      </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -2550,8 +2707,29 @@
       <c r="X21" s="77">
         <v>110</v>
       </c>
+      <c r="Y21" s="77">
+        <v>3.84</v>
+      </c>
+      <c r="Z21" s="77">
+        <v>1.0099</v>
+      </c>
+      <c r="AA21" s="77">
+        <v>137</v>
+      </c>
+      <c r="AB21" s="77">
+        <v>63.34</v>
+      </c>
+      <c r="AC21" s="77">
+        <v>12.082800000000001</v>
+      </c>
+      <c r="AD21" s="77">
+        <v>1970</v>
+      </c>
+      <c r="AE21" s="77" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -2610,8 +2788,30 @@
       <c r="X22" s="77">
         <v>191</v>
       </c>
+      <c r="Y22" s="77">
+        <v>4.18</v>
+      </c>
+      <c r="Z22" s="77">
+        <v>0.87560000000000004</v>
+      </c>
+      <c r="AA22" s="77">
+        <v>135</v>
+      </c>
+      <c r="AB22" s="77">
+        <f>60.98+0.62</f>
+        <v>61.599999999999994</v>
+      </c>
+      <c r="AC22" s="77">
+        <v>9.5932999999999993</v>
+      </c>
+      <c r="AD22" s="77">
+        <v>976.6</v>
+      </c>
+      <c r="AE22" s="77" t="s">
+        <v>48</v>
+      </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -2662,8 +2862,29 @@
       <c r="X23" s="77">
         <v>566</v>
       </c>
+      <c r="Y23" s="77">
+        <v>4.7</v>
+      </c>
+      <c r="Z23" s="77">
+        <v>0.9617</v>
+      </c>
+      <c r="AA23" s="77">
+        <v>117</v>
+      </c>
+      <c r="AB23" s="77">
+        <v>56.13</v>
+      </c>
+      <c r="AC23" s="77">
+        <v>10.324999999999999</v>
+      </c>
+      <c r="AD23" s="77">
+        <v>1405.3</v>
+      </c>
+      <c r="AE23" s="77" t="s">
+        <v>49</v>
+      </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -2704,8 +2925,30 @@
       <c r="V24" s="80"/>
       <c r="W24" s="80"/>
       <c r="X24" s="84"/>
+      <c r="Y24" s="84">
+        <v>6.1</v>
+      </c>
+      <c r="Z24" s="84">
+        <v>0.83899999999999997</v>
+      </c>
+      <c r="AA24" s="84">
+        <v>121</v>
+      </c>
+      <c r="AB24" s="84">
+        <f>46.77+0.83</f>
+        <v>47.6</v>
+      </c>
+      <c r="AC24" s="84">
+        <v>9.7091999999999992</v>
+      </c>
+      <c r="AD24" s="84">
+        <v>1347.49</v>
+      </c>
+      <c r="AE24" s="84" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -2746,8 +2989,29 @@
       <c r="V25" s="80"/>
       <c r="W25" s="80"/>
       <c r="X25" s="84"/>
+      <c r="Y25" s="84">
+        <v>2.7</v>
+      </c>
+      <c r="Z25" s="84">
+        <v>0.55459999999999998</v>
+      </c>
+      <c r="AA25" s="84">
+        <v>158</v>
+      </c>
+      <c r="AB25" s="84">
+        <v>69.430000000000007</v>
+      </c>
+      <c r="AC25" s="84">
+        <v>12.512700000000001</v>
+      </c>
+      <c r="AD25" s="84">
+        <v>1340.09</v>
+      </c>
+      <c r="AE25" s="84" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -2788,8 +3052,29 @@
       <c r="V26" s="80"/>
       <c r="W26" s="80"/>
       <c r="X26" s="84"/>
+      <c r="Y26" s="84">
+        <v>1.64</v>
+      </c>
+      <c r="Z26" s="84">
+        <v>0.4622</v>
+      </c>
+      <c r="AA26" s="84">
+        <v>120</v>
+      </c>
+      <c r="AB26" s="84">
+        <v>45.52</v>
+      </c>
+      <c r="AC26" s="84">
+        <v>7.8204000000000002</v>
+      </c>
+      <c r="AD26" s="84">
+        <v>1229.77</v>
+      </c>
+      <c r="AE26" s="84" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -2830,8 +3115,29 @@
       <c r="V27" s="80"/>
       <c r="W27" s="80"/>
       <c r="X27" s="84"/>
+      <c r="Y27" s="84">
+        <v>3.3</v>
+      </c>
+      <c r="Z27" s="84">
+        <v>0.39300000000000002</v>
+      </c>
+      <c r="AA27" s="84">
+        <v>69</v>
+      </c>
+      <c r="AB27" s="84">
+        <v>43.58</v>
+      </c>
+      <c r="AC27" s="84">
+        <v>5.5315000000000003</v>
+      </c>
+      <c r="AD27" s="84">
+        <v>1411.55</v>
+      </c>
+      <c r="AE27" s="84" t="s">
+        <v>53</v>
+      </c>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -2890,8 +3196,29 @@
       <c r="X28" s="93">
         <v>808</v>
       </c>
+      <c r="Y28" s="93">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="Z28" s="93">
+        <v>0.60680000000000001</v>
+      </c>
+      <c r="AA28" s="93">
+        <v>116</v>
+      </c>
+      <c r="AB28" s="93">
+        <v>59.53</v>
+      </c>
+      <c r="AC28" s="93">
+        <v>10.5433</v>
+      </c>
+      <c r="AD28" s="93">
+        <v>1313.02</v>
+      </c>
+      <c r="AE28" s="93" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -2950,8 +3277,29 @@
       <c r="X29" s="93">
         <v>668</v>
       </c>
+      <c r="Y29" s="93">
+        <v>3.97</v>
+      </c>
+      <c r="Z29" s="93">
+        <v>1.089</v>
+      </c>
+      <c r="AA29" s="93">
+        <v>142</v>
+      </c>
+      <c r="AB29" s="93">
+        <v>60.27</v>
+      </c>
+      <c r="AC29" s="93">
+        <v>13.506399999999999</v>
+      </c>
+      <c r="AD29" s="93">
+        <v>1361.88</v>
+      </c>
+      <c r="AE29" s="93" t="s">
+        <v>55</v>
+      </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -3010,8 +3358,29 @@
       <c r="X30" s="93">
         <v>920</v>
       </c>
+      <c r="Y30" s="93">
+        <v>6.33</v>
+      </c>
+      <c r="Z30" s="93">
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="AA30" s="93">
+        <v>85</v>
+      </c>
+      <c r="AB30" s="93">
+        <v>39.89</v>
+      </c>
+      <c r="AC30" s="93">
+        <v>11.229100000000001</v>
+      </c>
+      <c r="AD30" s="93">
+        <v>1263.72</v>
+      </c>
+      <c r="AE30" s="93" t="s">
+        <v>56</v>
+      </c>
     </row>
-    <row r="31" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -3070,8 +3439,29 @@
       <c r="X31" s="103">
         <v>130</v>
       </c>
+      <c r="Y31" s="103">
+        <v>3.41</v>
+      </c>
+      <c r="Z31" s="103">
+        <v>0.50919999999999999</v>
+      </c>
+      <c r="AA31" s="103">
+        <v>71</v>
+      </c>
+      <c r="AB31" s="103">
+        <v>53.12</v>
+      </c>
+      <c r="AC31" s="103">
+        <v>6.9410999999999996</v>
+      </c>
+      <c r="AD31" s="103">
+        <v>1253.58</v>
+      </c>
+      <c r="AE31" s="103" t="s">
+        <v>57</v>
+      </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -3132,8 +3522,29 @@
       <c r="X32" s="111">
         <v>150</v>
       </c>
+      <c r="Y32" s="111">
+        <v>2.38</v>
+      </c>
+      <c r="Z32" s="111">
+        <v>0.74480000000000002</v>
+      </c>
+      <c r="AA32" s="111">
+        <v>145</v>
+      </c>
+      <c r="AB32" s="111">
+        <v>55.63</v>
+      </c>
+      <c r="AC32" s="111">
+        <v>11.422000000000001</v>
+      </c>
+      <c r="AD32" s="111">
+        <v>1207.1500000000001</v>
+      </c>
+      <c r="AE32" s="111" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -3194,8 +3605,29 @@
       <c r="X33" s="119">
         <v>120</v>
       </c>
+      <c r="Y33" s="119">
+        <v>7.29</v>
+      </c>
+      <c r="Z33" s="119">
+        <v>0.81930000000000003</v>
+      </c>
+      <c r="AA33" s="119">
+        <v>109</v>
+      </c>
+      <c r="AB33" s="119">
+        <v>56.17</v>
+      </c>
+      <c r="AC33" s="119">
+        <v>9.0335999999999999</v>
+      </c>
+      <c r="AD33" s="119">
+        <v>1222.1400000000001</v>
+      </c>
+      <c r="AE33" s="119" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -3256,8 +3688,29 @@
       <c r="X34" s="119">
         <v>170</v>
       </c>
+      <c r="Y34" s="119">
+        <v>3.3</v>
+      </c>
+      <c r="Z34" s="119">
+        <v>0.89429999999999998</v>
+      </c>
+      <c r="AA34" s="119">
+        <v>117</v>
+      </c>
+      <c r="AB34" s="119">
+        <v>56.04</v>
+      </c>
+      <c r="AC34" s="119">
+        <v>10.404500000000001</v>
+      </c>
+      <c r="AD34" s="119">
+        <v>1093.95</v>
+      </c>
+      <c r="AE34" s="119" t="s">
+        <v>36</v>
+      </c>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -3310,8 +3763,29 @@
         <v>105</v>
       </c>
       <c r="X35" s="121"/>
+      <c r="Y35" s="121">
+        <v>4.22</v>
+      </c>
+      <c r="Z35" s="121">
+        <v>0.54300000000000004</v>
+      </c>
+      <c r="AA35" s="121">
+        <v>76</v>
+      </c>
+      <c r="AB35" s="121">
+        <v>40.119999999999997</v>
+      </c>
+      <c r="AC35" s="121">
+        <v>6.6025</v>
+      </c>
+      <c r="AD35" s="121">
+        <v>1343.07</v>
+      </c>
+      <c r="AE35" s="121" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -3354,8 +3828,29 @@
       <c r="V36" s="124"/>
       <c r="W36" s="123"/>
       <c r="X36" s="127"/>
+      <c r="Y36" s="127">
+        <v>8.61</v>
+      </c>
+      <c r="Z36" s="127">
+        <v>1.0141</v>
+      </c>
+      <c r="AA36" s="127">
+        <v>128</v>
+      </c>
+      <c r="AB36" s="127">
+        <v>69.31</v>
+      </c>
+      <c r="AC36" s="127">
+        <v>11.479200000000001</v>
+      </c>
+      <c r="AD36" s="127">
+        <v>1313.44</v>
+      </c>
+      <c r="AE36" s="127" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -3398,8 +3893,29 @@
       <c r="V37" s="124"/>
       <c r="W37" s="123"/>
       <c r="X37" s="127"/>
+      <c r="Y37" s="127">
+        <v>6.73</v>
+      </c>
+      <c r="Z37" s="127">
+        <v>0.90800000000000003</v>
+      </c>
+      <c r="AA37" s="127">
+        <v>112</v>
+      </c>
+      <c r="AB37" s="127">
+        <v>58.19</v>
+      </c>
+      <c r="AC37" s="127">
+        <v>9.5004000000000008</v>
+      </c>
+      <c r="AD37" s="127">
+        <v>1371.83</v>
+      </c>
+      <c r="AE37" s="127" t="s">
+        <v>39</v>
+      </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -3442,8 +3958,29 @@
       <c r="V38" s="124"/>
       <c r="W38" s="123"/>
       <c r="X38" s="127"/>
+      <c r="Y38" s="127">
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="Z38" s="127">
+        <v>0.51919999999999999</v>
+      </c>
+      <c r="AA38" s="127">
+        <v>127</v>
+      </c>
+      <c r="AB38" s="127">
+        <v>58.88</v>
+      </c>
+      <c r="AC38" s="127">
+        <v>11.9574</v>
+      </c>
+      <c r="AD38" s="127">
+        <v>1347.44</v>
+      </c>
+      <c r="AE38" s="127" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -3486,8 +4023,29 @@
       <c r="V39" s="124"/>
       <c r="W39" s="123"/>
       <c r="X39" s="127"/>
+      <c r="Y39" s="127">
+        <v>2.21</v>
+      </c>
+      <c r="Z39" s="127">
+        <v>0.59340000000000004</v>
+      </c>
+      <c r="AA39" s="127">
+        <v>110</v>
+      </c>
+      <c r="AB39" s="127">
+        <v>54.48</v>
+      </c>
+      <c r="AC39" s="127">
+        <v>9.8055000000000003</v>
+      </c>
+      <c r="AD39" s="127">
+        <v>1129.82</v>
+      </c>
+      <c r="AE39" s="127" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -3548,8 +4106,29 @@
       <c r="X40" s="139">
         <v>574</v>
       </c>
+      <c r="Y40" s="139">
+        <v>2.4</v>
+      </c>
+      <c r="Z40" s="139">
+        <v>0.61670000000000003</v>
+      </c>
+      <c r="AA40" s="139">
+        <v>138</v>
+      </c>
+      <c r="AB40" s="139">
+        <v>52.21</v>
+      </c>
+      <c r="AC40" s="139">
+        <v>11.1843</v>
+      </c>
+      <c r="AD40" s="139">
+        <v>1201.3</v>
+      </c>
+      <c r="AE40" s="139" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -3610,8 +4189,29 @@
       <c r="X41" s="139">
         <v>817</v>
       </c>
+      <c r="Y41" s="139">
+        <v>2.12</v>
+      </c>
+      <c r="Z41" s="139">
+        <v>0.60489999999999999</v>
+      </c>
+      <c r="AA41" s="139">
+        <v>134</v>
+      </c>
+      <c r="AB41" s="139">
+        <v>63.87</v>
+      </c>
+      <c r="AC41" s="139">
+        <v>12.145300000000001</v>
+      </c>
+      <c r="AD41" s="139">
+        <v>1280.06</v>
+      </c>
+      <c r="AE41" s="139" t="s">
+        <v>43</v>
+      </c>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -3672,8 +4272,29 @@
       <c r="X42" s="139">
         <v>751</v>
       </c>
+      <c r="Y42" s="139">
+        <v>2.8</v>
+      </c>
+      <c r="Z42" s="139">
+        <v>0.76349999999999996</v>
+      </c>
+      <c r="AA42" s="139">
+        <v>129</v>
+      </c>
+      <c r="AB42" s="139">
+        <v>62.27</v>
+      </c>
+      <c r="AC42" s="139">
+        <v>11.507</v>
+      </c>
+      <c r="AD42" s="139">
+        <v>1266.1500000000001</v>
+      </c>
+      <c r="AE42" s="139" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="43" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -3716,8 +4337,30 @@
       <c r="V43" s="147"/>
       <c r="W43" s="147"/>
       <c r="X43" s="148"/>
+      <c r="Y43" s="148">
+        <v>1.97</v>
+      </c>
+      <c r="Z43" s="148">
+        <v>0.67500000000000004</v>
+      </c>
+      <c r="AA43" s="148">
+        <v>125</v>
+      </c>
+      <c r="AB43" s="148">
+        <v>53.07</v>
+      </c>
+      <c r="AC43" s="148">
+        <v>10.924200000000001</v>
+      </c>
+      <c r="AD43" s="148">
+        <v>1274.79</v>
+      </c>
+      <c r="AE43" s="148" t="s">
+        <v>45</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
graf barras exploratorio in vivo
</commit_message>
<xml_diff>
--- a/BD Cobre.xlsx
+++ b/BD Cobre.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="35">
   <si>
     <t>id</t>
   </si>
@@ -123,76 +123,7 @@
     <t>adherido</t>
   </si>
   <si>
-    <t>506,21</t>
-  </si>
-  <si>
-    <t>166,65</t>
-  </si>
-  <si>
-    <t>330,50</t>
-  </si>
-  <si>
-    <t>317,26</t>
-  </si>
-  <si>
-    <t>151,55</t>
-  </si>
-  <si>
-    <t>202,84</t>
-  </si>
-  <si>
-    <t>553,50</t>
-  </si>
-  <si>
-    <t>510,23</t>
-  </si>
-  <si>
-    <t>499,54</t>
-  </si>
-  <si>
-    <t>602,80</t>
-  </si>
-  <si>
-    <t>451,20</t>
-  </si>
-  <si>
-    <t>646,10</t>
-  </si>
-  <si>
-    <t>283,64</t>
-  </si>
-  <si>
-    <t>512,02</t>
-  </si>
-  <si>
-    <t>232,64</t>
-  </si>
-  <si>
-    <t>298,00</t>
-  </si>
-  <si>
-    <t>219,90</t>
-  </si>
-  <si>
-    <t>495,33</t>
-  </si>
-  <si>
-    <t>748,86</t>
-  </si>
-  <si>
-    <t>426,74</t>
-  </si>
-  <si>
-    <t>569,88</t>
-  </si>
-  <si>
-    <t>342,04</t>
-  </si>
-  <si>
-    <t>198,64</t>
-  </si>
-  <si>
-    <t>366,62</t>
+    <t>EE</t>
   </si>
 </sst>
 </file>
@@ -1469,13 +1400,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE43"/>
+  <dimension ref="A1:AF43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1569,8 +1500,11 @@
       <c r="AE1" s="168" t="s">
         <v>33</v>
       </c>
+      <c r="AF1" s="168" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1626,7 +1560,7 @@
       <c r="W2" s="9"/>
       <c r="X2" s="11"/>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1668,7 +1602,7 @@
       <c r="W3" s="14"/>
       <c r="X3" s="15"/>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1710,7 +1644,7 @@
       <c r="W4" s="14"/>
       <c r="X4" s="15"/>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1766,7 +1700,7 @@
       <c r="W5" s="18"/>
       <c r="X5" s="20"/>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1822,7 +1756,7 @@
       <c r="W6" s="18"/>
       <c r="X6" s="20"/>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1878,7 +1812,7 @@
       <c r="W7" s="18"/>
       <c r="X7" s="20"/>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1934,7 +1868,7 @@
       <c r="W8" s="25"/>
       <c r="X8" s="26"/>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1990,7 +1924,7 @@
       <c r="W9" s="25"/>
       <c r="X9" s="26"/>
     </row>
-    <row r="10" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2046,7 +1980,7 @@
       <c r="W10" s="29"/>
       <c r="X10" s="30"/>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2106,7 +2040,7 @@
       <c r="W11" s="34"/>
       <c r="X11" s="36"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2166,7 +2100,7 @@
       <c r="W12" s="40"/>
       <c r="X12" s="42"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2208,7 +2142,7 @@
       <c r="W13" s="40"/>
       <c r="X13" s="42"/>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -2268,7 +2202,7 @@
       <c r="W14" s="46"/>
       <c r="X14" s="48"/>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -2328,7 +2262,7 @@
       <c r="W15" s="46"/>
       <c r="X15" s="48"/>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -2386,7 +2320,7 @@
       <c r="W16" s="46"/>
       <c r="X16" s="48"/>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -2446,7 +2380,7 @@
       <c r="W17" s="53"/>
       <c r="X17" s="55"/>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -2506,7 +2440,7 @@
       <c r="W18" s="53"/>
       <c r="X18" s="55"/>
     </row>
-    <row r="19" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -2566,7 +2500,7 @@
       <c r="W19" s="60"/>
       <c r="X19" s="62"/>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -2592,7 +2526,9 @@
         <v>37.5</v>
       </c>
       <c r="I20" s="64"/>
-      <c r="J20" s="67"/>
+      <c r="J20" s="67">
+        <v>0</v>
+      </c>
       <c r="K20" s="64"/>
       <c r="L20" s="64"/>
       <c r="M20" s="64"/>
@@ -2644,11 +2580,15 @@
       <c r="AD20" s="69">
         <v>1565.5</v>
       </c>
-      <c r="AE20" s="69" t="s">
-        <v>46</v>
+      <c r="AE20" s="69">
+        <v>283.64</v>
+      </c>
+      <c r="AF20">
+        <f>T20/Y20</f>
+        <v>3.3454545454545452</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -2674,7 +2614,9 @@
         <v>48.863636399999997</v>
       </c>
       <c r="I21" s="71"/>
-      <c r="J21" s="74"/>
+      <c r="J21" s="74">
+        <v>0</v>
+      </c>
       <c r="K21" s="71"/>
       <c r="L21" s="71"/>
       <c r="M21" s="71"/>
@@ -2725,11 +2667,15 @@
       <c r="AD21" s="77">
         <v>1970</v>
       </c>
-      <c r="AE21" s="77" t="s">
-        <v>47</v>
+      <c r="AE21" s="77">
+        <v>512.02</v>
+      </c>
+      <c r="AF21">
+        <f t="shared" ref="AF21:AF43" si="0">T21/Y21</f>
+        <v>4.661458333333333</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -2755,7 +2701,9 @@
         <v>20.454545499999998</v>
       </c>
       <c r="I22" s="71"/>
-      <c r="J22" s="74"/>
+      <c r="J22" s="74">
+        <v>0</v>
+      </c>
       <c r="K22" s="71"/>
       <c r="L22" s="71"/>
       <c r="M22" s="71"/>
@@ -2807,11 +2755,15 @@
       <c r="AD22" s="77">
         <v>976.6</v>
       </c>
-      <c r="AE22" s="77" t="s">
-        <v>48</v>
+      <c r="AE22" s="77">
+        <v>232.64</v>
+      </c>
+      <c r="AF22">
+        <f t="shared" si="0"/>
+        <v>12.129186602870815</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -2837,7 +2789,9 @@
         <v>37.5</v>
       </c>
       <c r="I23" s="71"/>
-      <c r="J23" s="74"/>
+      <c r="J23" s="74">
+        <v>0</v>
+      </c>
       <c r="K23" s="71"/>
       <c r="L23" s="71"/>
       <c r="M23" s="71"/>
@@ -2880,11 +2834,11 @@
       <c r="AD23" s="77">
         <v>1405.3</v>
       </c>
-      <c r="AE23" s="77" t="s">
-        <v>49</v>
+      <c r="AE23" s="77">
+        <v>298</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -2910,7 +2864,9 @@
         <v>42.045454599999999</v>
       </c>
       <c r="I24" s="80"/>
-      <c r="J24" s="83"/>
+      <c r="J24" s="83">
+        <v>0</v>
+      </c>
       <c r="K24" s="80"/>
       <c r="L24" s="80"/>
       <c r="M24" s="80"/>
@@ -2944,11 +2900,11 @@
       <c r="AD24" s="84">
         <v>1347.49</v>
       </c>
-      <c r="AE24" s="84" t="s">
-        <v>50</v>
+      <c r="AE24" s="84">
+        <v>219.9</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -2974,7 +2930,9 @@
         <v>51.136363699999997</v>
       </c>
       <c r="I25" s="80"/>
-      <c r="J25" s="83"/>
+      <c r="J25" s="83">
+        <v>0</v>
+      </c>
       <c r="K25" s="80"/>
       <c r="L25" s="80"/>
       <c r="M25" s="80"/>
@@ -3007,11 +2965,11 @@
       <c r="AD25" s="84">
         <v>1340.09</v>
       </c>
-      <c r="AE25" s="84" t="s">
-        <v>51</v>
+      <c r="AE25" s="84">
+        <v>495.33</v>
       </c>
     </row>
-    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -3037,7 +2995,9 @@
         <v>40.340909099999998</v>
       </c>
       <c r="I26" s="80"/>
-      <c r="J26" s="83"/>
+      <c r="J26" s="83">
+        <v>0</v>
+      </c>
       <c r="K26" s="80"/>
       <c r="L26" s="80"/>
       <c r="M26" s="80"/>
@@ -3070,11 +3030,11 @@
       <c r="AD26" s="84">
         <v>1229.77</v>
       </c>
-      <c r="AE26" s="84" t="s">
-        <v>52</v>
+      <c r="AE26" s="84">
+        <v>748.86</v>
       </c>
     </row>
-    <row r="27" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -3100,7 +3060,9 @@
         <v>40.340909099999998</v>
       </c>
       <c r="I27" s="80"/>
-      <c r="J27" s="83"/>
+      <c r="J27" s="83">
+        <v>0</v>
+      </c>
       <c r="K27" s="80"/>
       <c r="L27" s="80"/>
       <c r="M27" s="80"/>
@@ -3133,11 +3095,11 @@
       <c r="AD27" s="84">
         <v>1411.55</v>
       </c>
-      <c r="AE27" s="84" t="s">
-        <v>53</v>
+      <c r="AE27" s="84">
+        <v>426.74</v>
       </c>
     </row>
-    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -3163,7 +3125,9 @@
         <v>40.909090900000002</v>
       </c>
       <c r="I28" s="87"/>
-      <c r="J28" s="90"/>
+      <c r="J28" s="90">
+        <v>0</v>
+      </c>
       <c r="K28" s="87"/>
       <c r="L28" s="87"/>
       <c r="M28" s="87"/>
@@ -3214,11 +3178,15 @@
       <c r="AD28" s="93">
         <v>1313.02</v>
       </c>
-      <c r="AE28" s="93" t="s">
-        <v>54</v>
+      <c r="AE28" s="93">
+        <v>569.88</v>
+      </c>
+      <c r="AF28">
+        <f t="shared" si="0"/>
+        <v>13.391304347826088</v>
       </c>
     </row>
-    <row r="29" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -3244,7 +3212,9 @@
         <v>33.5227273</v>
       </c>
       <c r="I29" s="87"/>
-      <c r="J29" s="90"/>
+      <c r="J29" s="90">
+        <v>0</v>
+      </c>
       <c r="K29" s="87"/>
       <c r="L29" s="87"/>
       <c r="M29" s="87"/>
@@ -3295,11 +3265,15 @@
       <c r="AD29" s="93">
         <v>1361.88</v>
       </c>
-      <c r="AE29" s="93" t="s">
-        <v>55</v>
+      <c r="AE29" s="93">
+        <v>342.04</v>
+      </c>
+      <c r="AF29">
+        <f t="shared" si="0"/>
+        <v>9.7732997481108299</v>
       </c>
     </row>
-    <row r="30" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -3325,7 +3299,9 @@
         <v>39.7727273</v>
       </c>
       <c r="I30" s="87"/>
-      <c r="J30" s="90"/>
+      <c r="J30" s="90">
+        <v>0</v>
+      </c>
       <c r="K30" s="87"/>
       <c r="L30" s="87"/>
       <c r="M30" s="87"/>
@@ -3376,11 +3352,15 @@
       <c r="AD30" s="93">
         <v>1263.72</v>
       </c>
-      <c r="AE30" s="93" t="s">
-        <v>56</v>
+      <c r="AE30" s="93">
+        <v>198.64</v>
+      </c>
+      <c r="AF30">
+        <f t="shared" si="0"/>
+        <v>2.8120063191153237</v>
       </c>
     </row>
-    <row r="31" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -3406,7 +3386,9 @@
         <v>39.7727273</v>
       </c>
       <c r="I31" s="99"/>
-      <c r="J31" s="100"/>
+      <c r="J31" s="100">
+        <v>0</v>
+      </c>
       <c r="K31" s="96"/>
       <c r="L31" s="96"/>
       <c r="M31" s="96"/>
@@ -3457,11 +3439,15 @@
       <c r="AD31" s="103">
         <v>1253.58</v>
       </c>
-      <c r="AE31" s="103" t="s">
-        <v>57</v>
+      <c r="AE31" s="103">
+        <v>366.62</v>
+      </c>
+      <c r="AF31">
+        <f t="shared" si="0"/>
+        <v>10.293255131964809</v>
       </c>
     </row>
-    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -3540,11 +3526,15 @@
       <c r="AD32" s="111">
         <v>1207.1500000000001</v>
       </c>
-      <c r="AE32" s="111" t="s">
-        <v>34</v>
+      <c r="AE32" s="111">
+        <v>506.21</v>
+      </c>
+      <c r="AF32">
+        <f t="shared" si="0"/>
+        <v>6.6386554621848743</v>
       </c>
     </row>
-    <row r="33" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -3623,11 +3613,15 @@
       <c r="AD33" s="119">
         <v>1222.1400000000001</v>
       </c>
-      <c r="AE33" s="119" t="s">
-        <v>35</v>
+      <c r="AE33" s="119">
+        <v>166.65</v>
+      </c>
+      <c r="AF33">
+        <f t="shared" si="0"/>
+        <v>3.4156378600823043</v>
       </c>
     </row>
-    <row r="34" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -3706,11 +3700,15 @@
       <c r="AD34" s="119">
         <v>1093.95</v>
       </c>
-      <c r="AE34" s="119" t="s">
-        <v>36</v>
+      <c r="AE34" s="119">
+        <v>330.5</v>
+      </c>
+      <c r="AF34">
+        <f t="shared" si="0"/>
+        <v>4.1515151515151514</v>
       </c>
     </row>
-    <row r="35" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -3781,11 +3779,15 @@
       <c r="AD35" s="121">
         <v>1343.07</v>
       </c>
-      <c r="AE35" s="121" t="s">
-        <v>37</v>
+      <c r="AE35" s="121">
+        <v>317.26</v>
+      </c>
+      <c r="AF35">
+        <f t="shared" si="0"/>
+        <v>7.890995260663507</v>
       </c>
     </row>
-    <row r="36" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -3846,11 +3848,11 @@
       <c r="AD36" s="127">
         <v>1313.44</v>
       </c>
-      <c r="AE36" s="127" t="s">
-        <v>38</v>
+      <c r="AE36" s="127">
+        <v>151.55000000000001</v>
       </c>
     </row>
-    <row r="37" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -3911,11 +3913,11 @@
       <c r="AD37" s="127">
         <v>1371.83</v>
       </c>
-      <c r="AE37" s="127" t="s">
-        <v>39</v>
+      <c r="AE37" s="127">
+        <v>202.84</v>
       </c>
     </row>
-    <row r="38" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -3976,11 +3978,11 @@
       <c r="AD38" s="127">
         <v>1347.44</v>
       </c>
-      <c r="AE38" s="127" t="s">
-        <v>40</v>
+      <c r="AE38" s="127">
+        <v>553.5</v>
       </c>
     </row>
-    <row r="39" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -4041,11 +4043,11 @@
       <c r="AD39" s="127">
         <v>1129.82</v>
       </c>
-      <c r="AE39" s="127" t="s">
-        <v>41</v>
+      <c r="AE39" s="127">
+        <v>510.23</v>
       </c>
     </row>
-    <row r="40" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -4124,11 +4126,15 @@
       <c r="AD40" s="139">
         <v>1201.3</v>
       </c>
-      <c r="AE40" s="139" t="s">
-        <v>42</v>
+      <c r="AE40" s="139">
+        <v>499.54</v>
+      </c>
+      <c r="AF40">
+        <f t="shared" si="0"/>
+        <v>11.666666666666668</v>
       </c>
     </row>
-    <row r="41" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -4207,11 +4213,15 @@
       <c r="AD41" s="139">
         <v>1280.06</v>
       </c>
-      <c r="AE41" s="139" t="s">
-        <v>43</v>
+      <c r="AE41" s="139">
+        <v>602.79999999999995</v>
+      </c>
+      <c r="AF41">
+        <f t="shared" si="0"/>
+        <v>17.40566037735849</v>
       </c>
     </row>
-    <row r="42" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -4290,11 +4300,15 @@
       <c r="AD42" s="139">
         <v>1266.1500000000001</v>
       </c>
-      <c r="AE42" s="139" t="s">
-        <v>44</v>
+      <c r="AE42" s="139">
+        <v>451.2</v>
+      </c>
+      <c r="AF42">
+        <f t="shared" si="0"/>
+        <v>10.571428571428573</v>
       </c>
     </row>
-    <row r="43" spans="1:31" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:32" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -4355,8 +4369,8 @@
       <c r="AD43" s="148">
         <v>1274.79</v>
       </c>
-      <c r="AE43" s="148" t="s">
-        <v>45</v>
+      <c r="AE43" s="148">
+        <v>646.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modelos con observaciones VIVO
</commit_message>
<xml_diff>
--- a/BD Cobre.xlsx
+++ b/BD Cobre.xlsx
@@ -1,18 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julip\GitHub\Cobre\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF981FB-2CC2-4AA7-802E-13AB12B2D646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="236"/>
+    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="236" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -135,7 +152,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -627,7 +644,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="165">
+  <cellXfs count="164">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1107,14 +1124,13 @@
     <xf numFmtId="2" fontId="4" fillId="14" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1384,14 +1400,14 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AG43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1489,13 +1505,13 @@
       <c r="AD1" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="AE1" s="163" t="s">
+      <c r="AE1" t="s">
         <v>32</v>
       </c>
-      <c r="AF1" s="163" t="s">
+      <c r="AF1" t="s">
         <v>33</v>
       </c>
-      <c r="AG1" s="163" t="s">
+      <c r="AG1" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2582,7 +2598,7 @@
         <f>T20/Y20</f>
         <v>3.3454545454545452</v>
       </c>
-      <c r="AG20" s="164">
+      <c r="AG20" s="163">
         <f>Z20+AC20</f>
         <v>13.714399999999999</v>
       </c>
@@ -2673,7 +2689,7 @@
         <f t="shared" ref="AF21:AF42" si="0">T21/Y21</f>
         <v>4.661458333333333</v>
       </c>
-      <c r="AG21" s="164">
+      <c r="AG21" s="163">
         <f t="shared" ref="AG21:AG43" si="1">Z21+AC21</f>
         <v>13.092700000000001</v>
       </c>
@@ -2765,7 +2781,7 @@
         <f t="shared" si="0"/>
         <v>12.129186602870815</v>
       </c>
-      <c r="AG22" s="164">
+      <c r="AG22" s="163">
         <f t="shared" si="1"/>
         <v>10.4689</v>
       </c>
@@ -2844,7 +2860,7 @@
       <c r="AE23" s="72">
         <v>298</v>
       </c>
-      <c r="AG23" s="164">
+      <c r="AG23" s="163">
         <f t="shared" si="1"/>
         <v>11.2867</v>
       </c>
@@ -2914,7 +2930,7 @@
       <c r="AE24" s="79">
         <v>219.9</v>
       </c>
-      <c r="AG24" s="164">
+      <c r="AG24" s="163">
         <f t="shared" si="1"/>
         <v>10.5482</v>
       </c>
@@ -2983,7 +2999,7 @@
       <c r="AE25" s="79">
         <v>495.33</v>
       </c>
-      <c r="AG25" s="164">
+      <c r="AG25" s="163">
         <f t="shared" si="1"/>
         <v>13.067300000000001</v>
       </c>
@@ -3052,7 +3068,7 @@
       <c r="AE26" s="79">
         <v>748.86</v>
       </c>
-      <c r="AG26" s="164">
+      <c r="AG26" s="163">
         <f t="shared" si="1"/>
         <v>8.2826000000000004</v>
       </c>
@@ -3121,7 +3137,7 @@
       <c r="AE27" s="79">
         <v>426.74</v>
       </c>
-      <c r="AG27" s="164">
+      <c r="AG27" s="163">
         <f t="shared" si="1"/>
         <v>5.9245000000000001</v>
       </c>
@@ -3212,7 +3228,7 @@
         <f t="shared" si="0"/>
         <v>13.391304347826088</v>
       </c>
-      <c r="AG28" s="164">
+      <c r="AG28" s="163">
         <f t="shared" si="1"/>
         <v>11.1501</v>
       </c>
@@ -3303,7 +3319,7 @@
         <f t="shared" si="0"/>
         <v>9.7732997481108299</v>
       </c>
-      <c r="AG29" s="164">
+      <c r="AG29" s="163">
         <f t="shared" si="1"/>
         <v>14.5954</v>
       </c>
@@ -3394,7 +3410,7 @@
         <f t="shared" si="0"/>
         <v>2.8120063191153237</v>
       </c>
-      <c r="AG30" s="164">
+      <c r="AG30" s="163">
         <f t="shared" si="1"/>
         <v>12.234100000000002</v>
       </c>
@@ -3485,7 +3501,7 @@
         <f t="shared" si="0"/>
         <v>10.293255131964809</v>
       </c>
-      <c r="AG31" s="164">
+      <c r="AG31" s="163">
         <f t="shared" si="1"/>
         <v>7.4502999999999995</v>
       </c>
@@ -3576,7 +3592,7 @@
         <f t="shared" si="0"/>
         <v>6.6386554621848743</v>
       </c>
-      <c r="AG32" s="164">
+      <c r="AG32" s="163">
         <f t="shared" si="1"/>
         <v>12.1668</v>
       </c>
@@ -3667,7 +3683,7 @@
         <f t="shared" si="0"/>
         <v>3.4156378600823043</v>
       </c>
-      <c r="AG33" s="164">
+      <c r="AG33" s="163">
         <f t="shared" si="1"/>
         <v>9.8529</v>
       </c>
@@ -3758,7 +3774,7 @@
         <f t="shared" si="0"/>
         <v>4.1515151515151514</v>
       </c>
-      <c r="AG34" s="164">
+      <c r="AG34" s="163">
         <f t="shared" si="1"/>
         <v>11.2988</v>
       </c>
@@ -3841,7 +3857,7 @@
         <f t="shared" si="0"/>
         <v>7.890995260663507</v>
       </c>
-      <c r="AG35" s="164">
+      <c r="AG35" s="163">
         <f t="shared" si="1"/>
         <v>7.1455000000000002</v>
       </c>
@@ -3910,7 +3926,7 @@
       <c r="AE36" s="122">
         <v>151.55000000000001</v>
       </c>
-      <c r="AG36" s="164">
+      <c r="AG36" s="163">
         <f t="shared" si="1"/>
         <v>12.493300000000001</v>
       </c>
@@ -3979,7 +3995,7 @@
       <c r="AE37" s="122">
         <v>202.84</v>
       </c>
-      <c r="AG37" s="164">
+      <c r="AG37" s="163">
         <f t="shared" si="1"/>
         <v>10.4084</v>
       </c>
@@ -4048,7 +4064,7 @@
       <c r="AE38" s="122">
         <v>553.5</v>
       </c>
-      <c r="AG38" s="164">
+      <c r="AG38" s="163">
         <f t="shared" si="1"/>
         <v>12.476599999999999</v>
       </c>
@@ -4117,7 +4133,7 @@
       <c r="AE39" s="122">
         <v>510.23</v>
       </c>
-      <c r="AG39" s="164">
+      <c r="AG39" s="163">
         <f t="shared" si="1"/>
         <v>10.398900000000001</v>
       </c>
@@ -4208,7 +4224,7 @@
         <f t="shared" si="0"/>
         <v>11.666666666666668</v>
       </c>
-      <c r="AG40" s="164">
+      <c r="AG40" s="163">
         <f t="shared" si="1"/>
         <v>11.801</v>
       </c>
@@ -4299,7 +4315,7 @@
         <f t="shared" si="0"/>
         <v>17.40566037735849</v>
       </c>
-      <c r="AG41" s="164">
+      <c r="AG41" s="163">
         <f t="shared" si="1"/>
         <v>12.750200000000001</v>
       </c>
@@ -4390,7 +4406,7 @@
         <f t="shared" si="0"/>
         <v>10.571428571428573</v>
       </c>
-      <c r="AG42" s="164">
+      <c r="AG42" s="163">
         <f t="shared" si="1"/>
         <v>12.2705</v>
       </c>
@@ -4459,7 +4475,7 @@
       <c r="AE43" s="143">
         <v>646.1</v>
       </c>
-      <c r="AG43" s="164">
+      <c r="AG43" s="163">
         <f t="shared" si="1"/>
         <v>11.599200000000002</v>
       </c>

</xml_diff>